<commit_message>
added DateTime, DateOny and TimeOnly parsing
</commit_message>
<xml_diff>
--- a/FriendlyExcel.Tests/test-data-time/test.xlsx
+++ b/FriendlyExcel.Tests/test-data-time/test.xlsx
@@ -8,15 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
-    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
-    <sheet name="Лист3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
   <si>
     <t>Тест 1</t>
   </si>
@@ -103,6 +101,9 @@
   </si>
   <si>
     <t>Даты</t>
+  </si>
+  <si>
+    <t>Время</t>
   </si>
 </sst>
 </file>
@@ -146,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +159,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -459,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -469,9 +471,10 @@
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="16.6640625" customWidth="1"/>
     <col min="7" max="7" width="18.6640625" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -493,8 +496,11 @@
       <c r="G1" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -516,8 +522,11 @@
       <c r="G2" s="4">
         <v>45932</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" s="5">
+        <v>0.45833333333333331</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -539,8 +548,11 @@
       <c r="G3" s="4">
         <v>45933</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="5">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -562,8 +574,11 @@
       <c r="G4" s="4">
         <v>45934</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" s="5">
+        <v>0.54166666666666696</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -585,8 +600,11 @@
       <c r="G5" s="4">
         <v>45935</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="5">
+        <v>0.58333333333333304</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -608,8 +626,11 @@
       <c r="G6" s="4">
         <v>45936</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" s="5">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -631,8 +652,11 @@
       <c r="G7" s="4">
         <v>45937</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" s="5">
+        <v>0.66666666666666596</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -654,8 +678,11 @@
       <c r="G8" s="4">
         <v>45938</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" s="5">
+        <v>0.70833333333333304</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -677,8 +704,11 @@
       <c r="G9" s="4">
         <v>45939</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9" s="5">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -700,8 +730,11 @@
       <c r="G10" s="4">
         <v>45940</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H10" s="5">
+        <v>0.79166666666666596</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -723,197 +756,12 @@
       <c r="G11" s="4">
         <v>45941</v>
       </c>
+      <c r="H11" s="5">
+        <v>0.83333333333333304</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2">
-        <v>100</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2">
-        <v>200</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="3">
-        <v>1.2</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2">
-        <v>300</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="3">
-        <v>1.3</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2">
-        <v>400</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="3">
-        <v>1.4</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2">
-        <v>500</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2">
-        <v>600</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="3">
-        <v>1.6</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="2">
-        <v>700</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="3">
-        <v>1.7</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="2">
-        <v>800</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="3">
-        <v>1.8</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="2">
-        <v>900</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="3">
-        <v>1.9</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="2">
-        <v>1000</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="3">
-        <v>2</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>